<commit_message>
requirements-register: first version, evals; History and Updates tabs in the register template
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JEt3XhtRwUHbEHNFmAvqPW
</commit_message>
<xml_diff>
--- a/templates-source/discovery-setup/requirements-register.xlsx
+++ b/templates-source/discovery-setup/requirements-register.xlsx
@@ -8,6 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="History" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Updates" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -509,4 +511,136 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Req ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Version</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Replaced on</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Why it changed</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Conflicts</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>